<commit_message>
update bao dam quan y
</commit_message>
<xml_diff>
--- a/Resources/Sheet/Book2.xlsx
+++ b/Resources/Sheet/Book2.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\BODOIAPP\Resources\Sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196B5BB5-7B88-45D6-A964-55CDE961D6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D6E142-7F0C-42A9-85A5-F1DDBE98538A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuaChua" sheetId="7" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="8" r:id="rId2"/>
+    <sheet name="BaoDamQuanY" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
kh bao dam quan y
</commit_message>
<xml_diff>
--- a/Resources/Sheet/Book2.xlsx
+++ b/Resources/Sheet/Book2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\BODOIAPP\Resources\Sheet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\BODOIAPP\Resources\Sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{957FCAC1-1DFD-4F0B-B02E-1954116D9074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A65D87-F26B-4B2C-BBC7-99C41E8488E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuaChua" sheetId="7" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="44">
   <si>
     <t>Lựu đạn</t>
   </si>
@@ -450,6 +450,43 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -486,43 +523,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -799,48 +799,48 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A12AC3B-8D90-4B0D-96EA-52FB68143200}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="17"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="30"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="10"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="20"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="33"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="11"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1246,82 +1246,82 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C04A3E4-2F16-400C-90BF-200CB05E84C8}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="24" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="24" t="s">
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="21" t="s">
+      <c r="I2" s="16"/>
+      <c r="J2" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="21" t="s">
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="21" t="s">
+      <c r="G3" s="16"/>
+      <c r="H3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="22"/>
+      <c r="J3" s="14"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
       <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
       <c r="J4" s="4" t="s">
         <v>29</v>
       </c>
@@ -1624,105 +1624,105 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AC69830-15C2-40EF-A85C-0B734C645A25}">
   <dimension ref="A1:M12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="27" t="s">
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="L1" s="28"/>
-      <c r="M1" s="29"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="21"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="23"/>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="24" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="24" t="s">
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="21" t="s">
+      <c r="I2" s="16"/>
+      <c r="J2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="30" t="s">
+      <c r="K2" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="L2" s="30" t="s">
+      <c r="L2" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="M2" s="30" t="s">
+      <c r="M2" s="10" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="23"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="21" t="s">
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="21" t="s">
+      <c r="G3" s="16"/>
+      <c r="H3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="22"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="31"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
       <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
       <c r="J4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="32"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="32"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="5">
@@ -1759,15 +1759,15 @@
         <f>E5+I5</f>
         <v>0</v>
       </c>
-      <c r="K5" s="33">
+      <c r="K5" s="9">
         <f>ROUNDUP(J5/2,0)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="33">
+      <c r="L5" s="9">
         <f>J5-K5</f>
         <v>0</v>
       </c>
-      <c r="M5" s="33">
+      <c r="M5" s="9">
         <f>J5</f>
         <v>0</v>
       </c>
@@ -1779,17 +1779,40 @@
       <c r="B6" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="5"/>
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="6">
+        <f t="shared" ref="E6:E11" si="0">ROUND(C6*D6/100,0)</f>
+        <v>0</v>
+      </c>
       <c r="F6" s="8"/>
-      <c r="G6" s="5"/>
+      <c r="G6" s="6">
+        <f t="shared" ref="G6:G11" si="1">ROUND(E6*F6/100,0)</f>
+        <v>0</v>
+      </c>
       <c r="H6" s="8"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="33"/>
-      <c r="M6" s="33"/>
+      <c r="I6" s="6">
+        <f t="shared" ref="I6:I11" si="2">ROUND(H6*C6/100,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <f t="shared" ref="J6:J11" si="3">E6+I6</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="9">
+        <f t="shared" ref="K6:K11" si="4">ROUNDUP(J6/2,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="9">
+        <f t="shared" ref="L6:L11" si="5">J6-K6</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="9">
+        <f t="shared" ref="M6:M11" si="6">J6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:13" ht="24">
       <c r="A7" s="5" t="s">
@@ -1798,85 +1821,208 @@
       <c r="B7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="5"/>
+      <c r="C7" s="6">
+        <v>0</v>
+      </c>
       <c r="D7" s="8"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F7" s="8"/>
-      <c r="G7" s="5"/>
+      <c r="G7" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="H7" s="8"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-    </row>
-    <row r="8" spans="1:13">
+      <c r="I7" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K7" s="9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L7" s="9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M7" s="9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="24">
       <c r="A8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="B8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0</v>
+      </c>
       <c r="D8" s="8"/>
-      <c r="E8" s="5"/>
+      <c r="E8" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F8" s="8"/>
-      <c r="G8" s="5"/>
+      <c r="G8" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="H8" s="8"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
-      <c r="M8" s="33"/>
-    </row>
-    <row r="9" spans="1:13">
+      <c r="I8" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K8" s="9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L8" s="9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M8" s="9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="24">
       <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+      <c r="B9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0</v>
+      </c>
       <c r="D9" s="8"/>
-      <c r="E9" s="5"/>
+      <c r="E9" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F9" s="8"/>
-      <c r="G9" s="5"/>
+      <c r="G9" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="H9" s="8"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="I9" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K9" s="9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L9" s="9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M9" s="9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="24">
       <c r="A10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
+      <c r="B10" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0</v>
+      </c>
       <c r="D10" s="8"/>
-      <c r="E10" s="5"/>
+      <c r="E10" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F10" s="8"/>
-      <c r="G10" s="5"/>
+      <c r="G10" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="H10" s="8"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="33"/>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
+      <c r="I10" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K10" s="9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L10" s="9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M10" s="9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0</v>
+      </c>
       <c r="D11" s="8"/>
-      <c r="E11" s="5"/>
+      <c r="E11" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="F11" s="8"/>
-      <c r="G11" s="5"/>
+      <c r="G11" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="H11" s="8"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="33"/>
-      <c r="L11" s="33"/>
-      <c r="M11" s="33"/>
+      <c r="I11" s="6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="9">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="L11" s="9">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M11" s="9">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:13" ht="24">
       <c r="A12" s="5">
@@ -1901,18 +2047,12 @@
       <c r="H12" s="8"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="M2:M4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="B1:B4"/>
     <mergeCell ref="C1:C4"/>
@@ -1923,6 +2063,12 @@
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K4"/>
     <mergeCell ref="L2:L4"/>
+    <mergeCell ref="M2:M4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>